<commit_message>
Merge category coverage fix with Pharmaceuticals/Ultra Aggressive pct updates
- Preserve: 'Pharmaceuticals' added to US Equity Mid Cap (all tiers);
  Ultra Aggressive US Equity Small Cap 7.5%->8%, Non-US Equity
  Emerging Markets 7.5%->7%
- Re-apply: Corporate Bond, Multistrategy, Options Trading, Relative
  Value Arbitrage, Systematic Trend, Tactical Allocation -> Other
  Fixed Income; Global Allocation, Global Large-Stock Growth -> Non-US
  Equity Large Cap; Health, Utilities -> US Equity Mid Cap;
  Target-Date Retirement -> US Equity Large Cap (all tiers)
- Fix comma bug in Ultra Aggressive Other Fixed Income list
</commit_message>
<xml_diff>
--- a/First_Trust_Funds.xlsx
+++ b/First_Trust_Funds.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimpellizeri/Desktop/Aspire/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7A00593-4D36-9D45-AA8B-1C0F0B75FB7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{930FE0DF-B243-A945-A844-4CBF5BC883B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11000" yWindow="660" windowWidth="23560" windowHeight="19920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="53240" yWindow="600" windowWidth="23560" windowHeight="19920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -43,13 +43,21 @@
         <r>
           <rPr>
             <sz val="12"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Joseph Impellizeri:
-Source: First Trust Portfolios (official), https://www.ftportfolios.com/retail/etf/etfsummary.aspx?Ticker=AFLG</t>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Joseph Impellizeri:
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: First Trust Portfolios (official), https://www.ftportfolios.com/retail/etf/etfsummary.aspx?Ticker=AFLG</t>
         </r>
       </text>
     </comment>
@@ -868,7 +876,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -890,6 +898,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1250,6 +1264,28 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{175EA224-A1CD-544F-9520-DBF5F4E7B983}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;1aeac8b9-cab5-496a-ac56-333b80032943&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M32"/>

</xml_diff>